<commit_message>
Fixed age groups and borders in start list + schedule
</commit_message>
<xml_diff>
--- a/local/agegroups/2026-VWS2.xlsx
+++ b/local/agegroups/2026-VWS2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/agegroups/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E729EC5-C6AC-8143-9A77-70A9CCD5B917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525C41A8-00FC-4F48-B5E2-9C6B5F573C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17500" yWindow="2440" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24500" yWindow="3240" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="276">
   <si>
     <t>code</t>
   </si>
@@ -285,9 +285,6 @@
     <t>DEFAULT</t>
   </si>
   <si>
-    <t>QPoints</t>
-  </si>
-  <si>
     <t>ADH U11</t>
   </si>
   <si>
@@ -868,12 +865,6 @@
   </si>
   <si>
     <t>!WSO M100</t>
-  </si>
-  <si>
-    <t>QYouth</t>
-  </si>
-  <si>
-    <t>QMasters</t>
   </si>
 </sst>
 </file>
@@ -3466,10 +3457,10 @@
     </row>
     <row r="46" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
@@ -3522,10 +3513,10 @@
     </row>
     <row r="47" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
@@ -3579,10 +3570,10 @@
     </row>
     <row r="48" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
@@ -3632,10 +3623,10 @@
     </row>
     <row r="49" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
@@ -3683,10 +3674,10 @@
     </row>
     <row r="50" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
@@ -3734,10 +3725,10 @@
     </row>
     <row r="51" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
@@ -3783,10 +3774,10 @@
     </row>
     <row r="52" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
@@ -3834,10 +3825,10 @@
     </row>
     <row r="53" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
@@ -3885,10 +3876,10 @@
     </row>
     <row r="54" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
@@ -3936,10 +3927,10 @@
     </row>
     <row r="55" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
@@ -3987,10 +3978,10 @@
     </row>
     <row r="56" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
@@ -4038,10 +4029,10 @@
     </row>
     <row r="57" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>7</v>
@@ -4089,10 +4080,10 @@
     </row>
     <row r="58" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>7</v>
@@ -4140,10 +4131,10 @@
     </row>
     <row r="59" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>7</v>
@@ -4191,10 +4182,10 @@
     </row>
     <row r="60" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
@@ -4242,10 +4233,10 @@
     </row>
     <row r="61" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>7</v>
@@ -4293,10 +4284,10 @@
     </row>
     <row r="62" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>7</v>
@@ -4344,10 +4335,10 @@
     </row>
     <row r="63" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>7</v>
@@ -4395,10 +4386,10 @@
     </row>
     <row r="64" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>7</v>
@@ -4446,10 +4437,10 @@
     </row>
     <row r="65" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>7</v>
@@ -4497,10 +4488,10 @@
     </row>
     <row r="66" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>28</v>
@@ -4553,10 +4544,10 @@
     </row>
     <row r="67" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>28</v>
@@ -4610,10 +4601,10 @@
     </row>
     <row r="68" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>28</v>
@@ -4664,10 +4655,10 @@
     </row>
     <row r="69" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>28</v>
@@ -4715,10 +4706,10 @@
     </row>
     <row r="70" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>28</v>
@@ -4766,10 +4757,10 @@
     </row>
     <row r="71" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>28</v>
@@ -4817,10 +4808,10 @@
     </row>
     <row r="72" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>28</v>
@@ -4868,10 +4859,10 @@
     </row>
     <row r="73" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>28</v>
@@ -4918,10 +4909,10 @@
     </row>
     <row r="74" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>28</v>
@@ -4968,10 +4959,10 @@
     </row>
     <row r="75" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>28</v>
@@ -5018,10 +5009,10 @@
     </row>
     <row r="76" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>28</v>
@@ -5068,10 +5059,10 @@
     </row>
     <row r="77" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>28</v>
@@ -5118,10 +5109,10 @@
     </row>
     <row r="78" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>28</v>
@@ -5168,10 +5159,10 @@
     </row>
     <row r="79" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>28</v>
@@ -5218,10 +5209,10 @@
     </row>
     <row r="80" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>28</v>
@@ -5268,10 +5259,10 @@
     </row>
     <row r="81" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>28</v>
@@ -5318,10 +5309,10 @@
     </row>
     <row r="82" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A82" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>28</v>
@@ -5368,10 +5359,10 @@
     </row>
     <row r="83" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A83" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>28</v>
@@ -5418,10 +5409,10 @@
     </row>
     <row r="84" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A84" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>28</v>
@@ -5468,10 +5459,10 @@
     </row>
     <row r="85" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>28</v>
@@ -5518,10 +5509,10 @@
     </row>
     <row r="86" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A86" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>28</v>
@@ -5568,10 +5559,10 @@
     </row>
     <row r="87" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>7</v>
@@ -5624,10 +5615,10 @@
     </row>
     <row r="88" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>7</v>
@@ -5681,10 +5672,10 @@
     </row>
     <row r="89" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>7</v>
@@ -5734,10 +5725,10 @@
     </row>
     <row r="90" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>7</v>
@@ -5785,10 +5776,10 @@
     </row>
     <row r="91" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>7</v>
@@ -5836,10 +5827,10 @@
     </row>
     <row r="92" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>7</v>
@@ -5885,10 +5876,10 @@
     </row>
     <row r="93" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>7</v>
@@ -5936,10 +5927,10 @@
     </row>
     <row r="94" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>7</v>
@@ -5987,10 +5978,10 @@
     </row>
     <row r="95" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>7</v>
@@ -6038,10 +6029,10 @@
     </row>
     <row r="96" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>7</v>
@@ -6089,10 +6080,10 @@
     </row>
     <row r="97" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>7</v>
@@ -6140,10 +6131,10 @@
     </row>
     <row r="98" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>7</v>
@@ -6191,10 +6182,10 @@
     </row>
     <row r="99" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>7</v>
@@ -6242,10 +6233,10 @@
     </row>
     <row r="100" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>7</v>
@@ -6293,10 +6284,10 @@
     </row>
     <row r="101" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>7</v>
@@ -6344,10 +6335,10 @@
     </row>
     <row r="102" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>7</v>
@@ -6395,10 +6386,10 @@
     </row>
     <row r="103" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>7</v>
@@ -6446,10 +6437,10 @@
     </row>
     <row r="104" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>7</v>
@@ -6497,10 +6488,10 @@
     </row>
     <row r="105" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>7</v>
@@ -6548,10 +6539,10 @@
     </row>
     <row r="106" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>7</v>
@@ -6599,10 +6590,10 @@
     </row>
     <row r="107" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>28</v>
@@ -6655,10 +6646,10 @@
     </row>
     <row r="108" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>28</v>
@@ -6712,10 +6703,10 @@
     </row>
     <row r="109" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>28</v>
@@ -6766,10 +6757,10 @@
     </row>
     <row r="110" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>28</v>
@@ -6817,10 +6808,10 @@
     </row>
     <row r="111" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>28</v>
@@ -6868,10 +6859,10 @@
     </row>
     <row r="112" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>28</v>
@@ -6919,10 +6910,10 @@
     </row>
     <row r="113" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>28</v>
@@ -6970,10 +6961,10 @@
     </row>
     <row r="114" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>28</v>
@@ -7020,10 +7011,10 @@
     </row>
     <row r="115" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>28</v>
@@ -7070,10 +7061,10 @@
     </row>
     <row r="116" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>28</v>
@@ -7120,10 +7111,10 @@
     </row>
     <row r="117" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>28</v>
@@ -7170,10 +7161,10 @@
     </row>
     <row r="118" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>28</v>
@@ -7220,10 +7211,10 @@
     </row>
     <row r="119" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>28</v>
@@ -7270,10 +7261,10 @@
     </row>
     <row r="120" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>28</v>
@@ -7320,10 +7311,10 @@
     </row>
     <row r="121" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>28</v>
@@ -7370,10 +7361,10 @@
     </row>
     <row r="122" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>28</v>
@@ -7420,10 +7411,10 @@
     </row>
     <row r="123" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A123" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>28</v>
@@ -7470,10 +7461,10 @@
     </row>
     <row r="124" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A124" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>28</v>
@@ -7520,10 +7511,10 @@
     </row>
     <row r="125" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A125" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>28</v>
@@ -7570,10 +7561,10 @@
     </row>
     <row r="126" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A126" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>28</v>
@@ -7620,10 +7611,10 @@
     </row>
     <row r="127" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A127" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>28</v>
@@ -7670,10 +7661,10 @@
     </row>
     <row r="128" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>7</v>
@@ -7726,10 +7717,10 @@
     </row>
     <row r="129" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>7</v>
@@ -7783,10 +7774,10 @@
     </row>
     <row r="130" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>7</v>
@@ -7836,10 +7827,10 @@
     </row>
     <row r="131" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>7</v>
@@ -7887,10 +7878,10 @@
     </row>
     <row r="132" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>7</v>
@@ -7938,10 +7929,10 @@
     </row>
     <row r="133" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>7</v>
@@ -7987,10 +7978,10 @@
     </row>
     <row r="134" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>7</v>
@@ -8038,10 +8029,10 @@
     </row>
     <row r="135" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>7</v>
@@ -8089,10 +8080,10 @@
     </row>
     <row r="136" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>7</v>
@@ -8140,10 +8131,10 @@
     </row>
     <row r="137" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>7</v>
@@ -8191,10 +8182,10 @@
     </row>
     <row r="138" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>7</v>
@@ -8242,10 +8233,10 @@
     </row>
     <row r="139" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>7</v>
@@ -8293,10 +8284,10 @@
     </row>
     <row r="140" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>7</v>
@@ -8344,10 +8335,10 @@
     </row>
     <row r="141" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>7</v>
@@ -8395,10 +8386,10 @@
     </row>
     <row r="142" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>7</v>
@@ -8446,10 +8437,10 @@
     </row>
     <row r="143" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>7</v>
@@ -8497,10 +8488,10 @@
     </row>
     <row r="144" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>7</v>
@@ -8548,10 +8539,10 @@
     </row>
     <row r="145" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>7</v>
@@ -8599,10 +8590,10 @@
     </row>
     <row r="146" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>7</v>
@@ -8650,10 +8641,10 @@
     </row>
     <row r="147" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>7</v>
@@ -8701,10 +8692,10 @@
     </row>
     <row r="148" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>28</v>
@@ -8757,10 +8748,10 @@
     </row>
     <row r="149" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>28</v>
@@ -8814,10 +8805,10 @@
     </row>
     <row r="150" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>28</v>
@@ -8868,10 +8859,10 @@
     </row>
     <row r="151" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>28</v>
@@ -8919,10 +8910,10 @@
     </row>
     <row r="152" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>28</v>
@@ -8970,10 +8961,10 @@
     </row>
     <row r="153" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>28</v>
@@ -9021,10 +9012,10 @@
     </row>
     <row r="154" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>28</v>
@@ -9072,10 +9063,10 @@
     </row>
     <row r="155" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>28</v>
@@ -9122,10 +9113,10 @@
     </row>
     <row r="156" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>28</v>
@@ -9172,10 +9163,10 @@
     </row>
     <row r="157" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>28</v>
@@ -9222,10 +9213,10 @@
     </row>
     <row r="158" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>28</v>
@@ -9272,10 +9263,10 @@
     </row>
     <row r="159" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>28</v>
@@ -9322,10 +9313,10 @@
     </row>
     <row r="160" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>28</v>
@@ -9372,10 +9363,10 @@
     </row>
     <row r="161" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>28</v>
@@ -9422,10 +9413,10 @@
     </row>
     <row r="162" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>28</v>
@@ -9472,10 +9463,10 @@
     </row>
     <row r="163" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>28</v>
@@ -9522,10 +9513,10 @@
     </row>
     <row r="164" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A164" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>28</v>
@@ -9572,10 +9563,10 @@
     </row>
     <row r="165" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A165" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>28</v>
@@ -9622,10 +9613,10 @@
     </row>
     <row r="166" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A166" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>28</v>
@@ -9672,10 +9663,10 @@
     </row>
     <row r="167" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A167" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>28</v>
@@ -9722,10 +9713,10 @@
     </row>
     <row r="168" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A168" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>28</v>
@@ -9772,10 +9763,10 @@
     </row>
     <row r="169" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>7</v>
@@ -9828,10 +9819,10 @@
     </row>
     <row r="170" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>7</v>
@@ -9885,10 +9876,10 @@
     </row>
     <row r="171" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>7</v>
@@ -9938,10 +9929,10 @@
     </row>
     <row r="172" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>7</v>
@@ -9989,10 +9980,10 @@
     </row>
     <row r="173" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>7</v>
@@ -10040,10 +10031,10 @@
     </row>
     <row r="174" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>7</v>
@@ -10089,10 +10080,10 @@
     </row>
     <row r="175" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>7</v>
@@ -10140,10 +10131,10 @@
     </row>
     <row r="176" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>7</v>
@@ -10191,10 +10182,10 @@
     </row>
     <row r="177" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>7</v>
@@ -10242,10 +10233,10 @@
     </row>
     <row r="178" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>7</v>
@@ -10293,10 +10284,10 @@
     </row>
     <row r="179" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>7</v>
@@ -10344,10 +10335,10 @@
     </row>
     <row r="180" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>7</v>
@@ -10395,10 +10386,10 @@
     </row>
     <row r="181" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>7</v>
@@ -10446,10 +10437,10 @@
     </row>
     <row r="182" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>7</v>
@@ -10497,10 +10488,10 @@
     </row>
     <row r="183" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>7</v>
@@ -10548,10 +10539,10 @@
     </row>
     <row r="184" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>7</v>
@@ -10599,10 +10590,10 @@
     </row>
     <row r="185" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>7</v>
@@ -10650,10 +10641,10 @@
     </row>
     <row r="186" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>7</v>
@@ -10701,10 +10692,10 @@
     </row>
     <row r="187" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>7</v>
@@ -10752,10 +10743,10 @@
     </row>
     <row r="188" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>7</v>
@@ -10803,10 +10794,10 @@
     </row>
     <row r="189" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>28</v>
@@ -10859,10 +10850,10 @@
     </row>
     <row r="190" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>28</v>
@@ -10916,10 +10907,10 @@
     </row>
     <row r="191" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>28</v>
@@ -10970,10 +10961,10 @@
     </row>
     <row r="192" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>28</v>
@@ -11021,10 +11012,10 @@
     </row>
     <row r="193" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>28</v>
@@ -11072,10 +11063,10 @@
     </row>
     <row r="194" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>28</v>
@@ -11123,10 +11114,10 @@
     </row>
     <row r="195" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>28</v>
@@ -11174,10 +11165,10 @@
     </row>
     <row r="196" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>28</v>
@@ -11224,10 +11215,10 @@
     </row>
     <row r="197" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>28</v>
@@ -11274,10 +11265,10 @@
     </row>
     <row r="198" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>28</v>
@@ -11324,10 +11315,10 @@
     </row>
     <row r="199" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>28</v>
@@ -11374,10 +11365,10 @@
     </row>
     <row r="200" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>28</v>
@@ -11424,10 +11415,10 @@
     </row>
     <row r="201" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>28</v>
@@ -11474,10 +11465,10 @@
     </row>
     <row r="202" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>28</v>
@@ -11524,10 +11515,10 @@
     </row>
     <row r="203" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C203" s="1" t="s">
         <v>28</v>
@@ -11574,10 +11565,10 @@
     </row>
     <row r="204" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C204" s="1" t="s">
         <v>28</v>
@@ -11624,10 +11615,10 @@
     </row>
     <row r="205" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A205" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C205" s="1" t="s">
         <v>28</v>
@@ -11674,10 +11665,10 @@
     </row>
     <row r="206" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A206" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C206" s="1" t="s">
         <v>28</v>
@@ -11724,10 +11715,10 @@
     </row>
     <row r="207" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A207" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C207" s="1" t="s">
         <v>28</v>
@@ -11774,10 +11765,10 @@
     </row>
     <row r="208" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A208" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C208" s="1" t="s">
         <v>28</v>
@@ -11824,10 +11815,10 @@
     </row>
     <row r="209" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A209" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>28</v>
@@ -11874,10 +11865,10 @@
     </row>
     <row r="210" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B210" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="B210" s="1" t="s">
-        <v>240</v>
       </c>
       <c r="C210" s="1" t="s">
         <v>7</v>
@@ -11926,10 +11917,10 @@
     </row>
     <row r="211" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C211" s="1" t="s">
         <v>7</v>
@@ -11979,10 +11970,10 @@
     </row>
     <row r="212" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C212" s="1" t="s">
         <v>7</v>
@@ -12028,10 +12019,10 @@
     </row>
     <row r="213" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C213" s="1" t="s">
         <v>7</v>
@@ -12075,10 +12066,10 @@
     </row>
     <row r="214" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B214" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="B214" s="1" t="s">
-        <v>245</v>
       </c>
       <c r="C214" s="1" t="s">
         <v>7</v>
@@ -12120,10 +12111,10 @@
     </row>
     <row r="215" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B215" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="B215" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="C215" s="1" t="s">
         <v>7</v>
@@ -12165,10 +12156,10 @@
     </row>
     <row r="216" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B216" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="B216" s="1" t="s">
-        <v>240</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>28</v>
@@ -12219,10 +12210,10 @@
     </row>
     <row r="217" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C217" s="1" t="s">
         <v>28</v>
@@ -12273,10 +12264,10 @@
     </row>
     <row r="218" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C218" s="1" t="s">
         <v>28</v>
@@ -12324,10 +12315,10 @@
     </row>
     <row r="219" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C219" s="1" t="s">
         <v>28</v>
@@ -12372,10 +12363,10 @@
     </row>
     <row r="220" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B220" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="B220" s="1" t="s">
-        <v>245</v>
       </c>
       <c r="C220" s="1" t="s">
         <v>28</v>
@@ -12417,10 +12408,10 @@
     </row>
     <row r="221" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B221" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="B221" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="C221" s="1" t="s">
         <v>28</v>
@@ -12462,10 +12453,10 @@
     </row>
     <row r="222" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B222" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="B222" s="1" t="s">
-        <v>249</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>7</v>
@@ -12507,10 +12498,10 @@
     </row>
     <row r="223" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C223" s="1" t="s">
         <v>7</v>
@@ -12552,10 +12543,10 @@
     </row>
     <row r="224" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C224" s="1" t="s">
         <v>7</v>
@@ -12597,10 +12588,10 @@
     </row>
     <row r="225" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C225" s="1" t="s">
         <v>7</v>
@@ -12642,10 +12633,10 @@
     </row>
     <row r="226" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C226" s="1" t="s">
         <v>7</v>
@@ -12687,10 +12678,10 @@
     </row>
     <row r="227" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C227" s="1" t="s">
         <v>7</v>
@@ -12732,10 +12723,10 @@
     </row>
     <row r="228" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C228" s="1" t="s">
         <v>7</v>
@@ -12777,10 +12768,10 @@
     </row>
     <row r="229" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C229" s="1" t="s">
         <v>7</v>
@@ -12822,10 +12813,10 @@
     </row>
     <row r="230" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C230" s="1" t="s">
         <v>7</v>
@@ -12867,10 +12858,10 @@
     </row>
     <row r="231" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C231" s="1" t="s">
         <v>7</v>
@@ -12912,10 +12903,10 @@
     </row>
     <row r="232" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C232" s="1" t="s">
         <v>7</v>
@@ -12957,10 +12948,10 @@
     </row>
     <row r="233" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C233" s="1" t="s">
         <v>7</v>
@@ -13002,10 +12993,10 @@
     </row>
     <row r="234" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C234" s="1" t="s">
         <v>7</v>
@@ -13047,10 +13038,10 @@
     </row>
     <row r="235" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C235" s="1" t="s">
         <v>7</v>
@@ -13092,10 +13083,10 @@
     </row>
     <row r="236" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>28</v>
@@ -13137,10 +13128,10 @@
     </row>
     <row r="237" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C237" s="1" t="s">
         <v>28</v>
@@ -13182,10 +13173,10 @@
     </row>
     <row r="238" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C238" s="1" t="s">
         <v>28</v>
@@ -13227,10 +13218,10 @@
     </row>
     <row r="239" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C239" s="1" t="s">
         <v>28</v>
@@ -13272,10 +13263,10 @@
     </row>
     <row r="240" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>28</v>
@@ -13317,10 +13308,10 @@
     </row>
     <row r="241" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>28</v>
@@ -13362,10 +13353,10 @@
     </row>
     <row r="242" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C242" s="1" t="s">
         <v>28</v>
@@ -13407,10 +13398,10 @@
     </row>
     <row r="243" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C243" s="1" t="s">
         <v>28</v>
@@ -13452,10 +13443,10 @@
     </row>
     <row r="244" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C244" s="1" t="s">
         <v>28</v>
@@ -13497,10 +13488,10 @@
     </row>
     <row r="245" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C245" s="1" t="s">
         <v>28</v>
@@ -13542,10 +13533,10 @@
     </row>
     <row r="246" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C246" s="1" t="s">
         <v>28</v>
@@ -13587,10 +13578,10 @@
     </row>
     <row r="247" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C247" s="1" t="s">
         <v>28</v>
@@ -13632,10 +13623,10 @@
     </row>
     <row r="248" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C248" s="1" t="s">
         <v>28</v>
@@ -13677,10 +13668,10 @@
     </row>
     <row r="249" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C249" s="1" t="s">
         <v>28</v>
@@ -13831,7 +13822,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>79</v>
@@ -13882,13 +13873,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>82</v>
+      <c r="F3" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="I3">
         <v>28</v>
@@ -13933,7 +13924,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>79</v>
@@ -13984,7 +13975,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>79</v>
@@ -14026,7 +14017,7 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>6</v>
@@ -14035,7 +14026,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>79</v>
@@ -14077,7 +14068,7 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>12</v>
@@ -14086,7 +14077,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>79</v>
@@ -14128,7 +14119,7 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>6</v>
@@ -14137,7 +14128,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>79</v>
@@ -14179,7 +14170,7 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>12</v>
@@ -14188,7 +14179,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>79</v>
@@ -14230,7 +14221,7 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A10" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>6</v>
@@ -14239,7 +14230,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>79</v>
@@ -14281,7 +14272,7 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A11" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>12</v>
@@ -14290,7 +14281,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>79</v>
@@ -14332,7 +14323,7 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>6</v>
@@ -14341,7 +14332,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>79</v>
@@ -14383,7 +14374,7 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A13" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>12</v>
@@ -14392,7 +14383,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>79</v>
@@ -14443,7 +14434,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>54</v>
@@ -14491,7 +14482,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>55</v>
@@ -14530,7 +14521,7 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A16" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>6</v>
@@ -14545,7 +14536,7 @@
         <v>79</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>277</v>
+        <v>53</v>
       </c>
       <c r="I16">
         <v>28</v>
@@ -14581,7 +14572,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.15">
       <c r="A17" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>12</v>
@@ -14596,7 +14587,7 @@
         <v>79</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>278</v>
+        <v>55</v>
       </c>
       <c r="I17">
         <v>28</v>

</xml_diff>